<commit_message>
fix: allow department-wide exit question imports without courses
</commit_message>
<xml_diff>
--- a/apps/quiz/static/quiz/exit_exam_import_template.xlsx
+++ b/apps/quiz/static/quiz/exit_exam_import_template.xlsx
@@ -514,10 +514,10 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="54" customHeight="1">
+    <row r="2" ht="75" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Required. Use active course name or code e.g. Data Structures &amp; Algorithms or CS202</t>
+          <t>Optional. Active course name or code; leave blank for department-wide questions. Saved as a topic tag; does not assign a course to the paper.</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -567,7 +567,7 @@
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>Optional comma separated tags e.g. arrays,basics</t>
+          <t>Optional comma separated topics for practice e.g. leadership,ethics. Course and chapter are not required.</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">

</xml_diff>

<commit_message>
feat: support optional sixth answer choice across quiz flows
</commit_message>
<xml_diff>
--- a/apps/quiz/static/quiz/exit_exam_import_template.xlsx
+++ b/apps/quiz/static/quiz/exit_exam_import_template.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:M2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -445,11 +445,12 @@
     <col width="28" customWidth="1" min="5" max="5"/>
     <col width="28" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="46" customWidth="1" min="9" max="9"/>
-    <col width="22" customWidth="1" min="10" max="10"/>
-    <col width="36" customWidth="1" min="11" max="11"/>
-    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="46" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="36" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -490,25 +491,30 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
+          <t>option_f</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
           <t>correct_option</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>explanation</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>difficulty</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>topic_tags</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>year_source</t>
         </is>
@@ -552,25 +558,30 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>a b c d or e</t>
+          <t>MCQ: optional 6th choice. Fill when correct_option is f.</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
+          <t>MCQ: a b c d e f | True/False: a or b</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
           <t>Shown to student after answering in practice mode</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>easy / medium / hard (default: medium)</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>Optional comma separated topics for practice e.g. leadership,ethics. Course and chapter are not required.</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t>Optional e.g. 2023</t>
         </is>

</xml_diff>